<commit_message>
remote updated from .bat file
</commit_message>
<xml_diff>
--- a/server-side/modelling/results/all all tables.xlsx
+++ b/server-side/modelling/results/all all tables.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="cueva_second_phase svm 1 0p1 cm" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="cueva_second_phase svm 1 0p1 metrics" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="cueva svm 1 0p1 cm" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="cueva svm 1 0p1 metrics" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="hossain gbt 600 0p1 5 cm" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="hossain gbt 600 0p1 5 metrics" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="hossain svm 10 0p1 cm" sheetId="5" state="visible" r:id="rId5"/>

</xml_diff>